<commit_message>
working model with more power plants
</commit_message>
<xml_diff>
--- a/Cost results.xlsx
+++ b/Cost results.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/laura_linuesa-domenech_tennet_eu/Documents/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E5E243D-321E-4FAE-956A-18B6A808E507}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E09D8B00-6638-4A24-AAED-619D8118F205}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{4AE1EDD8-8ACF-4AF9-86A6-B0088C54F040}"/>
+    <workbookView xWindow="2213" yWindow="0" windowWidth="14340" windowHeight="11003" activeTab="1" xr2:uid="{4AE1EDD8-8ACF-4AF9-86A6-B0088C54F040}"/>
   </bookViews>
   <sheets>
     <sheet name="clear_freq=1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="clear_freq=3" sheetId="3" r:id="rId2"/>
+    <sheet name="clear_freq=6" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="33">
   <si>
     <t>ECONOMIC SUMMARY</t>
   </si>
@@ -150,7 +151,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -187,6 +188,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -200,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -208,6 +215,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,27 +592,27 @@
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="8">
         <v>253500</v>
       </c>
-      <c r="C5" s="1">
-        <v>20610685.185185187</v>
-      </c>
-      <c r="D5" s="1">
-        <v>81.304478048067793</v>
+      <c r="C5" s="8">
+        <v>21022500</v>
+      </c>
+      <c r="D5">
+        <v>82.928994082840234</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1">
-        <v>29479.881716353604</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2947988.1716353605</v>
-      </c>
-      <c r="D6" s="1">
+      <c r="B6" s="8">
+        <v>29566.948707521442</v>
+      </c>
+      <c r="C6" s="8">
+        <v>2956694.8707521441</v>
+      </c>
+      <c r="D6">
         <v>100</v>
       </c>
     </row>
@@ -610,27 +620,26 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="8">
         <v>75650</v>
       </c>
-      <c r="C7" s="1">
-        <v>6153615.4320987649</v>
-      </c>
-      <c r="D7" s="1">
-        <v>81.343231091854136</v>
+      <c r="C7" s="8">
+        <v>6283200</v>
+      </c>
+      <c r="D7">
+        <v>83.056179775280896</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="1">
-        <v>358629.88171635359</v>
-      </c>
-      <c r="C8" s="1">
-        <v>29712288.788919311</v>
-      </c>
-      <c r="D8" s="1"/>
+      <c r="B8" s="8">
+        <v>358716.94870752143</v>
+      </c>
+      <c r="C8" s="8">
+        <v>30262394.870752145</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -659,53 +668,53 @@
       <c r="A12" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="1">
-        <v>21452219.566548292</v>
-      </c>
-      <c r="C12" s="1">
+      <c r="B12" s="8">
+        <v>21656807.854490768</v>
+      </c>
+      <c r="C12" s="8">
         <v>288000</v>
       </c>
-      <c r="D12" s="1">
-        <v>301441.49852552346</v>
+      <c r="D12" s="8">
+        <v>298828.06013357785</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="1">
-        <v>4545369.3826796887</v>
-      </c>
-      <c r="C13" s="1">
-        <v>34654.136187511845</v>
-      </c>
-      <c r="D13" s="1">
-        <v>517608.65505291609</v>
+      <c r="B13" s="8">
+        <v>4535375.1440216415</v>
+      </c>
+      <c r="C13" s="8">
+        <v>33849.436310376856</v>
+      </c>
+      <c r="D13" s="8">
+        <v>510857.45800521004</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="1">
-        <v>3038026.3825465213</v>
-      </c>
-      <c r="C14" s="1">
-        <v>84776.466675331365</v>
-      </c>
-      <c r="D14" s="1">
-        <v>744231.22046728164</v>
+      <c r="B14" s="8">
+        <v>2752470.5845989869</v>
+      </c>
+      <c r="C14" s="8">
+        <v>85889.430123734637</v>
+      </c>
+      <c r="D14" s="8">
+        <v>753356.57519324264</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="1">
-        <v>29035615.331774503</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
+      <c r="B15" s="8">
+        <v>28944653.583111398</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
@@ -718,7 +727,7 @@
       <c r="A18" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="8">
         <v>7605000</v>
       </c>
     </row>
@@ -726,15 +735,15 @@
       <c r="A19" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="1">
-        <v>2947988.1716353605</v>
+      <c r="B19" s="8">
+        <v>2956694.8707521441</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="8">
         <v>0</v>
       </c>
     </row>
@@ -742,16 +751,16 @@
       <c r="A21" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="1">
-        <v>10552988.17163536</v>
+      <c r="B21" s="8">
+        <v>10561694.870752145</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="1">
-        <v>62076.40100961976</v>
+      <c r="B22" s="8">
+        <v>62127.616886777323</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -765,32 +774,32 @@
       <c r="A25" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="1">
-        <v>13847219.566548292</v>
+      <c r="B25" s="8">
+        <v>14051807.854490768</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="1">
-        <v>1597381.2110443283</v>
+      <c r="B26" s="8">
+        <v>1578680.2732694973</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="1">
-        <v>3038026.3825465213</v>
+      <c r="B27" s="8">
+        <v>2752470.5845989869</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="1">
-        <v>18482627.16013914</v>
+      <c r="B28" s="8">
+        <v>18382958.712359253</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -803,70 +812,73 @@
       <c r="A31" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="1">
-        <v>4820.1182836463968</v>
+      <c r="B31" s="8">
+        <v>4733.0512924785617</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="1">
-        <v>5900.3688886258269</v>
+      <c r="B32" s="8">
+        <v>5930.4864860277967</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="1">
-        <v>96.824011139467771</v>
+      <c r="B33" s="8">
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>22</v>
       </c>
-      <c r="B34" s="1">
-        <v>56.041995114699134</v>
+      <c r="B34" s="8">
+        <v>59.931731593819194</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="1">
-        <v>466703.18638933101</v>
+      <c r="B35" s="8">
+        <v>473305.12924785615</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="1">
-        <v>330668.44443129137</v>
+      <c r="B36" s="8">
+        <v>355424.32430138986</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>25</v>
       </c>
-      <c r="B37" s="1">
-        <v>136034.74195803964</v>
+      <c r="B37" s="8">
+        <v>117880.80494646629</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="1">
-        <v>800.20436445905671</v>
+      <c r="B38" s="8">
+        <v>693.4164996850958</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="A40" s="7" t="s">
         <v>32</v>
       </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
@@ -886,13 +898,13 @@
       <c r="A42" t="s">
         <v>5</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42">
         <v>253500</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42">
         <v>253500</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42">
         <v>0</v>
       </c>
     </row>
@@ -900,13 +912,13 @@
       <c r="A43" t="s">
         <v>6</v>
       </c>
-      <c r="B43" s="1">
-        <v>29479.881716353604</v>
-      </c>
-      <c r="C43" s="1">
-        <v>29479.8817163536</v>
-      </c>
-      <c r="D43" s="1">
+      <c r="B43">
+        <v>29566.948707521442</v>
+      </c>
+      <c r="C43">
+        <v>29566.948707521442</v>
+      </c>
+      <c r="D43">
         <v>1.1368683772161603E-13</v>
       </c>
     </row>
@@ -914,14 +926,14 @@
       <c r="A44" t="s">
         <v>7</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44">
         <v>75650</v>
       </c>
-      <c r="C44" s="1">
+      <c r="C44">
         <v>75650</v>
       </c>
-      <c r="D44" s="1">
-        <v>2.2737367544323206E-13</v>
+      <c r="D44">
+        <v>1.1368683772161603E-13</v>
       </c>
     </row>
   </sheetData>
@@ -930,10 +942,989 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA8B9C3-C35E-4BF3-9CE3-A4FB113A9C65}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2752EBB7-9311-4CAE-82F2-5AE38C585B2F}">
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="25.73046875" customWidth="1"/>
+    <col min="2" max="2" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.265625" customWidth="1"/>
+    <col min="5" max="5" width="11.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="8">
+        <v>255000</v>
+      </c>
+      <c r="C5" s="8">
+        <v>20735592.592592593</v>
+      </c>
+      <c r="D5">
+        <v>81.316049382716045</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="8">
+        <v>29348.149876238378</v>
+      </c>
+      <c r="C6" s="8">
+        <v>2934814.9876238382</v>
+      </c>
+      <c r="D6">
+        <v>100.00000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="8">
+        <v>76104.991183523845</v>
+      </c>
+      <c r="C7" s="8">
+        <v>6239569.3429394215</v>
+      </c>
+      <c r="D7">
+        <v>81.986335533407711</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="8">
+        <v>360453.14105976222</v>
+      </c>
+      <c r="C8" s="8">
+        <v>29909976.923155852</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="8">
+        <v>22677112.668843187</v>
+      </c>
+      <c r="C12" s="8">
+        <v>286500.00000000006</v>
+      </c>
+      <c r="D12" s="8">
+        <v>287717.13021356007</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="8">
+        <v>3569220.6119229496</v>
+      </c>
+      <c r="C13" s="8">
+        <v>33685.806460712025</v>
+      </c>
+      <c r="D13" s="8">
+        <v>169077.54096673679</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="8">
+        <v>6015560.6160172746</v>
+      </c>
+      <c r="C14" s="8">
+        <v>85955.558416339933</v>
+      </c>
+      <c r="D14" s="8">
+        <v>280756.48043458001</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="8">
+        <v>32261893.896783412</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="9"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="8">
+        <v>7650000</v>
+      </c>
+      <c r="C18" s="8"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="8">
+        <v>2934814.9876238382</v>
+      </c>
+      <c r="C19" s="8"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="8">
+        <v>0</v>
+      </c>
+      <c r="C20" s="8"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="8">
+        <v>10584814.987623839</v>
+      </c>
+      <c r="C21" s="8"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="8">
+        <v>185698.5085548042</v>
+      </c>
+      <c r="C22" s="8"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="9"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="8">
+        <v>15027112.668843187</v>
+      </c>
+      <c r="C25" s="8"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="8">
+        <v>634405.62429911131</v>
+      </c>
+      <c r="C26" s="8"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="8">
+        <v>6015560.6160172746</v>
+      </c>
+      <c r="C27" s="8"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="8">
+        <v>21677078.909159571</v>
+      </c>
+      <c r="C28" s="8"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B29" s="8"/>
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="8">
+        <v>4861.4544484969874</v>
+      </c>
+      <c r="C31" s="8"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="8">
+        <v>6431.4828116847966</v>
+      </c>
+      <c r="C32" s="8"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33" s="8">
+        <v>100</v>
+      </c>
+      <c r="C33" s="8"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="8">
+        <v>50</v>
+      </c>
+      <c r="C34" s="8"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="8">
+        <v>486145.44484969875</v>
+      </c>
+      <c r="C35" s="8"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36" s="8">
+        <v>321574.14058423985</v>
+      </c>
+      <c r="C36" s="8"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" s="8">
+        <v>164571.30426545889</v>
+      </c>
+      <c r="C37" s="8"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" s="8">
+        <v>2887.2158643062962</v>
+      </c>
+      <c r="C38" s="8"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42">
+        <v>255000</v>
+      </c>
+      <c r="C42">
+        <v>255000</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>29348.149876238378</v>
+      </c>
+      <c r="C43">
+        <v>29348.149876238378</v>
+      </c>
+      <c r="D43">
+        <v>1.1368683772161603E-13</v>
+      </c>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44">
+        <v>76104.991183523845</v>
+      </c>
+      <c r="C44">
+        <v>76104.991183523845</v>
+      </c>
+      <c r="D44">
+        <v>1.1368683772161603E-13</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41F2AF54-2B1C-476A-8233-8C4B3C9DA612}">
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.73046875" customWidth="1"/>
+    <col min="2" max="2" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.265625" customWidth="1"/>
+    <col min="5" max="5" width="11.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="8">
+        <v>259500</v>
+      </c>
+      <c r="C5" s="8">
+        <v>20914092.592592593</v>
+      </c>
+      <c r="D5">
+        <v>80.593805751801895</v>
+      </c>
+      <c r="E5" s="8">
+        <v>259500</v>
+      </c>
+      <c r="F5" s="8">
+        <v>21053185.185185187</v>
+      </c>
+      <c r="G5">
+        <v>81.129808035395712</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="8">
+        <v>30700.633224201607</v>
+      </c>
+      <c r="C6" s="8">
+        <v>3070063.3224201608</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6" s="8">
+        <v>30129.497109504537</v>
+      </c>
+      <c r="F6" s="8">
+        <v>3012949.7109504556</v>
+      </c>
+      <c r="G6">
+        <v>100.00000000000007</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="8">
+        <v>76817.907613653049</v>
+      </c>
+      <c r="C7" s="8">
+        <v>6233400.3355996488</v>
+      </c>
+      <c r="D7">
+        <v>81.145146089500756</v>
+      </c>
+      <c r="E7" s="8">
+        <v>76706.102261776497</v>
+      </c>
+      <c r="F7" s="8">
+        <v>6301106.0148755545</v>
+      </c>
+      <c r="G7">
+        <v>82.146085240671468</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="8">
+        <v>367018.54083785467</v>
+      </c>
+      <c r="C8" s="8">
+        <v>30217556.250612404</v>
+      </c>
+      <c r="E8" s="8">
+        <v>366335.59937128105</v>
+      </c>
+      <c r="F8" s="8">
+        <v>30367240.911011197</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B9" s="8"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="8">
+        <v>22557019.731501672</v>
+      </c>
+      <c r="C12" s="8">
+        <v>286500.00000000006</v>
+      </c>
+      <c r="D12" s="8">
+        <v>286929.86713003926</v>
+      </c>
+      <c r="E12" s="8">
+        <v>23177446.686123695</v>
+      </c>
+      <c r="F12" s="8">
+        <v>286500</v>
+      </c>
+      <c r="G12" s="8">
+        <v>286660.49650383677</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="8">
+        <v>3626207.6627232404</v>
+      </c>
+      <c r="C13" s="8">
+        <v>34695.159424024918</v>
+      </c>
+      <c r="D13" s="8">
+        <v>97947.391636887871</v>
+      </c>
+      <c r="E13" s="8">
+        <v>3595345.4376449259</v>
+      </c>
+      <c r="F13" s="8">
+        <v>34425.469253956559</v>
+      </c>
+      <c r="G13" s="8">
+        <v>98004.846459071952</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="8">
+        <v>6351458.8745754492</v>
+      </c>
+      <c r="C14" s="8">
+        <v>85796.52924579625</v>
+      </c>
+      <c r="D14" s="8">
+        <v>175458.20222055708</v>
+      </c>
+      <c r="E14" s="8">
+        <v>6527993.1049968712</v>
+      </c>
+      <c r="F14" s="8">
+        <v>85425.448899664087</v>
+      </c>
+      <c r="G14" s="8">
+        <v>172302.3360018449</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="8">
+        <v>32534686.268800359</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8">
+        <v>33300785.228765491</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="9"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="8">
+        <v>7785000</v>
+      </c>
+      <c r="C18" s="8">
+        <v>7785000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="8">
+        <v>3070063.3224201608</v>
+      </c>
+      <c r="C19" s="8">
+        <v>3012949.7109504556</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="8">
+        <v>0</v>
+      </c>
+      <c r="C20" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="8">
+        <v>10855063.322420161</v>
+      </c>
+      <c r="C21" s="8">
+        <v>10797949.710950457</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="8">
+        <v>374312.52835931588</v>
+      </c>
+      <c r="C22" s="8">
+        <v>372343.09348105022</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="9"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="8">
+        <v>14772019.731501672</v>
+      </c>
+      <c r="C25" s="8">
+        <v>15392446.686123695</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="8">
+        <v>556144.34030307969</v>
+      </c>
+      <c r="C26" s="8">
+        <v>582395.72669447027</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="8">
+        <v>6351458.8745754492</v>
+      </c>
+      <c r="C27" s="8">
+        <v>6527993.1049968712</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="8">
+        <v>21679622.946380202</v>
+      </c>
+      <c r="C28" s="8">
+        <v>22502835.517815039</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="8">
+        <v>5008.4010759659523</v>
+      </c>
+      <c r="C31" s="8">
+        <v>4957.6511629892721</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="8">
+        <v>6701.1744840408164</v>
+      </c>
+      <c r="C32" s="8">
+        <v>6789.7510471552396</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33" s="8">
+        <v>99.630530110337986</v>
+      </c>
+      <c r="C33" s="8">
+        <v>99.302818490998504</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="8">
+        <v>50.132469019580618</v>
+      </c>
+      <c r="C34" s="8">
+        <v>50.355031377597243</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="8">
+        <v>498989.65420367499</v>
+      </c>
+      <c r="C35" s="8">
+        <v>492308.73358001129</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36" s="8">
+        <v>335946.42221598036</v>
+      </c>
+      <c r="C36" s="8">
+        <v>341898.12702557584</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" s="8">
+        <v>163043.23198769463</v>
+      </c>
+      <c r="C37" s="8">
+        <v>150410.60655443545</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" s="8">
+        <v>5622.1804133687801</v>
+      </c>
+      <c r="C38" s="8">
+        <v>5186.5726398081188</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42">
+        <v>259500</v>
+      </c>
+      <c r="C42">
+        <v>259500</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>259500</v>
+      </c>
+      <c r="F42">
+        <v>259500</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>30700.633224201607</v>
+      </c>
+      <c r="C43">
+        <v>30700.633224201607</v>
+      </c>
+      <c r="D43">
+        <v>1.1368683772161603E-13</v>
+      </c>
+      <c r="E43">
+        <v>30129.497109504537</v>
+      </c>
+      <c r="F43">
+        <v>30129.497109504537</v>
+      </c>
+      <c r="G43">
+        <v>5.6843418860808015E-14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44">
+        <v>76817.907613653049</v>
+      </c>
+      <c r="C44">
+        <v>76817.907613653049</v>
+      </c>
+      <c r="D44">
+        <v>1.1368683772161603E-13</v>
+      </c>
+      <c r="E44">
+        <v>76706.102261776497</v>
+      </c>
+      <c r="F44">
+        <v>76706.102261776497</v>
+      </c>
+      <c r="G44">
+        <v>1.1368683772161603E-13</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>